<commit_message>
fix: pozycje zawodnikow z section zamiast position, limit strzelcow 200
</commit_message>
<xml_diff>
--- a/data/krolowie_strzelcow.xlsx
+++ b/data/krolowie_strzelcow.xlsx
@@ -480,7 +480,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Offence</t>
         </is>
       </c>
     </row>
@@ -540,7 +540,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Right Winger</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Offence</t>
         </is>
       </c>
     </row>
@@ -700,7 +700,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Right Winger</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Revert "fix: pozycje zawodnikow z section zamiast position, limit strzelcow 200"
This reverts commit f1eee29495b08f37d462ffd987d73a3845bb6139.
</commit_message>
<xml_diff>
--- a/data/krolowie_strzelcow.xlsx
+++ b/data/krolowie_strzelcow.xlsx
@@ -480,7 +480,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Offence</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -540,7 +540,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Right Winger</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Offence</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -700,7 +700,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Right Winger</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>

</xml_diff>